<commit_message>
Laser DXF request list: assembly number in the title row, no extra sheet
- requestList.titleCell (default A2) gets the assembly number
  (requestList.title, default {ID}-{REV}, e.g. S180-06068-37005-1); the
  cell's formatting (merged, bordered row) is kept.
- The "DXF list" data sheet is no longer added by default
  (requestList.dataSheet = "" ; set a name to bring it back).
- Stand-in template gets the merged A2:D2 title row; tests check the
  title, the merge and the optional data sheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AA72gNxMn1Q6iyHah18D6U
</commit_message>
<xml_diff>
--- a/nx-laser-dxf/samples/request_list_example.xlsx
+++ b/nx-laser-dxf/samples/request_list_example.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jig Part Request List" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DXF list" sheetId="2" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Jig Part Request List'!$A$1:$D$37</definedName>
@@ -20,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,6 +30,9 @@
     <font>
       <sz val="16"/>
       <u val="single"/>
+    </font>
+    <font>
+      <sz val="14"/>
     </font>
     <font>
       <u val="single"/>
@@ -44,13 +46,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
     <border>
       <left style="thin"/>
@@ -62,19 +78,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -495,574 +516,333 @@
         <v/>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1"/>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S180-06068-37005-1</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n"/>
+      <c r="C2" s="5" t="n"/>
+      <c r="D2" s="6" t="n"/>
+    </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Part Number</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Thickness</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">S180-06068-47002-1</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">MILD STEEL</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">6mm</t>
         </is>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">S180-06068-47003-1</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">MILD STEEL</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">6mm</t>
         </is>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">S180-06068-47004-1</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">MILD STEEL</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">6mm</t>
         </is>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">S180-06068-47005-1</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">MILD STEEL</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">3mm</t>
         </is>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">S180-06068-47006-1</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">MILD STEEL</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">3mm</t>
         </is>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">S180-06068-47007-1</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">MILD STEEL</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">3mm</t>
         </is>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="8" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
+      <c r="A11" s="8" t="n"/>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
+      <c r="A13" s="8" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
+      <c r="A15" s="8" t="n"/>
+      <c r="B15" s="8" t="n"/>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
+      <c r="A16" s="8" t="n"/>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
+      <c r="A17" s="8" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
+      <c r="A18" s="8" t="n"/>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="8" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n"/>
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="8" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n"/>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
+      <c r="A20" s="8" t="n"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="n"/>
-      <c r="B21" s="5" t="n"/>
-      <c r="C21" s="5" t="n"/>
-      <c r="D21" s="5" t="n"/>
+      <c r="A21" s="8" t="n"/>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="8" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="n"/>
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="5" t="n"/>
-      <c r="D22" s="5" t="n"/>
+      <c r="A22" s="8" t="n"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="8" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="n"/>
-      <c r="B23" s="5" t="n"/>
-      <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
+      <c r="A23" s="8" t="n"/>
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="8" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="n"/>
-      <c r="B24" s="5" t="n"/>
-      <c r="C24" s="5" t="n"/>
-      <c r="D24" s="5" t="n"/>
+      <c r="A24" s="8" t="n"/>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="8" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="n"/>
-      <c r="B25" s="5" t="n"/>
-      <c r="C25" s="5" t="n"/>
-      <c r="D25" s="5" t="n"/>
+      <c r="A25" s="8" t="n"/>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="8" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="n"/>
-      <c r="B26" s="5" t="n"/>
-      <c r="C26" s="5" t="n"/>
-      <c r="D26" s="5" t="n"/>
+      <c r="A26" s="8" t="n"/>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="8" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="n"/>
-      <c r="B27" s="5" t="n"/>
-      <c r="C27" s="5" t="n"/>
-      <c r="D27" s="5" t="n"/>
+      <c r="A27" s="8" t="n"/>
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="8" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="n"/>
-      <c r="B28" s="5" t="n"/>
-      <c r="C28" s="5" t="n"/>
-      <c r="D28" s="5" t="n"/>
+      <c r="A28" s="8" t="n"/>
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="8" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="n"/>
-      <c r="B29" s="5" t="n"/>
-      <c r="C29" s="5" t="n"/>
-      <c r="D29" s="5" t="n"/>
+      <c r="A29" s="8" t="n"/>
+      <c r="B29" s="8" t="n"/>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="8" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="n"/>
-      <c r="B30" s="5" t="n"/>
-      <c r="C30" s="5" t="n"/>
-      <c r="D30" s="5" t="n"/>
+      <c r="A30" s="8" t="n"/>
+      <c r="B30" s="8" t="n"/>
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="8" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="n"/>
-      <c r="B31" s="5" t="n"/>
-      <c r="C31" s="5" t="n"/>
-      <c r="D31" s="5" t="n"/>
+      <c r="A31" s="8" t="n"/>
+      <c r="B31" s="8" t="n"/>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="8" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="n"/>
-      <c r="B32" s="5" t="n"/>
-      <c r="C32" s="5" t="n"/>
-      <c r="D32" s="5" t="n"/>
+      <c r="A32" s="8" t="n"/>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="8" t="n"/>
+      <c r="D32" s="8" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="n"/>
-      <c r="B33" s="5" t="n"/>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="5" t="n"/>
+      <c r="A33" s="8" t="n"/>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="8" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="n"/>
-      <c r="B34" s="5" t="n"/>
-      <c r="C34" s="5" t="n"/>
-      <c r="D34" s="5" t="n"/>
+      <c r="A34" s="8" t="n"/>
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="8" t="n"/>
+      <c r="D34" s="8" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="n"/>
-      <c r="B35" s="5" t="n"/>
-      <c r="C35" s="5" t="n"/>
-      <c r="D35" s="5" t="n"/>
+      <c r="A35" s="8" t="n"/>
+      <c r="B35" s="8" t="n"/>
+      <c r="C35" s="8" t="n"/>
+      <c r="D35" s="8" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="n"/>
-      <c r="B36" s="5" t="n"/>
-      <c r="C36" s="5" t="n"/>
-      <c r="D36" s="5" t="n"/>
+      <c r="A36" s="8" t="n"/>
+      <c r="B36" s="8" t="n"/>
+      <c r="C36" s="8" t="n"/>
+      <c r="D36" s="8" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="n"/>
-      <c r="B37" s="5" t="n"/>
-      <c r="C37" s="5" t="n"/>
-      <c r="D37" s="5" t="n"/>
+      <c r="A37" s="8" t="n"/>
+      <c r="B37" s="8" t="n"/>
+      <c r="C37" s="8" t="n"/>
+      <c r="D37" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="F1:G1"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="8" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="11" customWidth="1"/>
-    <col min="7" max="7" width="56" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ID</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Revision</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Name</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Qty</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Material</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Thickness</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DXF path</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">S180-06068-47002-1</t>
-        </is>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLATE 0 &amp; CO &lt;X&gt;</t>
-        </is>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MILD STEEL</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6mm</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C:\Laser DXF\S180-06068-37003-1\S180-06068-47002-1.dxf</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">S180-06068-47003-1</t>
-        </is>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLATE 1 &amp; CO &lt;X&gt;</t>
-        </is>
-      </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MILD STEEL</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6mm</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C:\Laser DXF\S180-06068-37003-1\S180-06068-47003-1.dxf</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">S180-06068-47004-1</t>
-        </is>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLATE 2 &amp; CO &lt;X&gt;</t>
-        </is>
-      </c>
-      <c r="D4">
-        <v>3</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MILD STEEL</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6mm</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C:\Laser DXF\S180-06068-37003-1\S180-06068-47004-1.dxf</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">S180-06068-47005-1</t>
-        </is>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLATE 3 &amp; CO &lt;X&gt;</t>
-        </is>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MILD STEEL</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3mm</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C:\Laser DXF\S180-06068-37003-1\S180-06068-47005-1.dxf</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">S180-06068-47006-1</t>
-        </is>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLATE 4 &amp; CO &lt;X&gt;</t>
-        </is>
-      </c>
-      <c r="D6">
-        <v>2</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MILD STEEL</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3mm</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C:\Laser DXF\S180-06068-37003-1\S180-06068-47006-1.dxf</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">S180-06068-47007-1</t>
-        </is>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLATE 5 &amp; CO &lt;X&gt;</t>
-        </is>
-      </c>
-      <c r="D7">
-        <v>3</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MILD STEEL</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3mm</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C:\Laser DXF\S180-06068-37003-1\S180-06068-47007-1.dxf</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Laser DXF request list: CSV data back as a second sheet
The workbook again has a "DXF list" sheet with the full CSV table (all
columns) after the populated front sheet; the CSV file is still written.
requestList.dataSheet = "" leaves it out.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AA72gNxMn1Q6iyHah18D6U
</commit_message>
<xml_diff>
--- a/nx-laser-dxf/samples/request_list_example.xlsx
+++ b/nx-laser-dxf/samples/request_list_example.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jig Part Request List" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DXF list" sheetId="2" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Jig Part Request List'!$A$1:$D$37</definedName>
@@ -845,4 +846,255 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="8" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
+    <col min="7" max="7" width="56" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Revision</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qty</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Material</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thickness</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DXF path</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S180-06068-47002-1</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLATE 0 &amp; CO &lt;X&gt;</t>
+        </is>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MILD STEEL</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6mm</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C:\Laser DXF\S180-06068-37003-1\S180-06068-47002-1.dxf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S180-06068-47003-1</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLATE 1 &amp; CO &lt;X&gt;</t>
+        </is>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MILD STEEL</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6mm</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C:\Laser DXF\S180-06068-37003-1\S180-06068-47003-1.dxf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S180-06068-47004-1</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLATE 2 &amp; CO &lt;X&gt;</t>
+        </is>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MILD STEEL</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6mm</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C:\Laser DXF\S180-06068-37003-1\S180-06068-47004-1.dxf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S180-06068-47005-1</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLATE 3 &amp; CO &lt;X&gt;</t>
+        </is>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MILD STEEL</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3mm</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C:\Laser DXF\S180-06068-37003-1\S180-06068-47005-1.dxf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S180-06068-47006-1</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLATE 4 &amp; CO &lt;X&gt;</t>
+        </is>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MILD STEEL</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3mm</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C:\Laser DXF\S180-06068-37003-1\S180-06068-47006-1.dxf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S180-06068-47007-1</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLATE 5 &amp; CO &lt;X&gt;</t>
+        </is>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MILD STEEL</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3mm</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C:\Laser DXF\S180-06068-37003-1\S180-06068-47007-1.dxf</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>